<commit_message>
Accreditamento FSE 2.0 RSA - aggiornamento test case v9.0.0 (data.json, checklist, PDF risultati)
</commit_message>
<xml_diff>
--- a/GATEWAY/S1#111#MEDITHYNKSRLXX/MEDITHYNK/ISYPATIENT/1.0.0/report-checklist_V9.0.0.xlsx
+++ b/GATEWAY/S1#111#MEDITHYNKSRLXX/MEDITHYNK/ISYPATIENT/1.0.0/report-checklist_V9.0.0.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ismae\it-fse-accreditamento\GATEWAY\S1#111#MEDITHYNKSRLXX\MEDITHYNK\ISYPATIENT\1.0.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E52B214-1824-4C33-8220-CEF8A68E77F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FC84620-BA91-4005-84D9-5D0ADE44C496}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Istruzioni Compilazione" sheetId="1" r:id="rId1"/>
@@ -2410,207 +2410,15 @@
 I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso nella sezione "CASO DI TEST 6" riportata nei documenti "casi di test Relazione CTC" e "CDA2_Relazione_CTC_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
   </si>
   <si>
-    <t>2026-03-25T09:36:33.2610000Z</t>
-  </si>
-  <si>
-    <t>a31de43d7a2698ecdb8a962c53c3af24</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.0714baf97a^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
     <t>Errore durante la validazione del CDA2</t>
   </si>
   <si>
     <t>Il documento viene salvato su Firebase con fseStatus=ERROR. Il medico può proseguire normalmente con il suo lavoro.</t>
   </si>
   <si>
-    <t>2026-03-25T09:39:55.7090000Z</t>
-  </si>
-  <si>
-    <t>6b9d72770853bfc8c02e0df78c4cab68</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.db105bc68f^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>2026-03-25T09:46:49.9660000Z</t>
-  </si>
-  <si>
-    <t>7c89d1de6bf7961cd8a77b08180c19af</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.ab2c4562e8^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>2026-03-25T09:48:59.7910000Z</t>
-  </si>
-  <si>
-    <t>ce193a66fde43652c4a2f45b5cb9ef9d</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.c9f6f49a16^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>2026-03-25T09:51:25.0190000Z</t>
-  </si>
-  <si>
-    <t>054727c128e4a33b2948e903f43a9600</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.1fdc042e84^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>2026-03-25T09:54:09.1980000Z</t>
-  </si>
-  <si>
-    <t>d215007584da915b6315764118aea98b</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.903cf86048^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>2026-03-25T09:55:29.1900000Z</t>
-  </si>
-  <si>
-    <t>9cde33ff37baa77a923eedbdd7ccb2a4</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.91d841b17c^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>2026-03-25T09:13:24.4150000Z</t>
-  </si>
-  <si>
-    <t>7ca07f957493ac63f2e1b9e643989c08</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.d964970dc8^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>2026-03-25T09:14:45.9230000Z</t>
-  </si>
-  <si>
-    <t>dc8c8cf9ea68acba51e58e237cab4794</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.053257c647^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>2026-03-25T09:57:40.4160000Z</t>
-  </si>
-  <si>
-    <t>9b3f3cc3b2867e505434f6cf1b7fc1bc</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.8b51a84326^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>2026-03-25T09:59:22.0360000Z</t>
-  </si>
-  <si>
-    <t>84fe4f5647a080f5fab232a11aee6c14</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.954ca6d0ee^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>2026-03-25T10:01:39.5780000Z</t>
-  </si>
-  <si>
-    <t>2cabf8dde62186d71ea434f6d12d3166</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.7672113dd1^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>2026-03-25T09:16:36.0920000Z</t>
-  </si>
-  <si>
-    <t>7fdbb2595200d90e9af3046e4d7dfcf3</t>
-  </si>
-  <si>
     <t>UNKNOWN_WORKFLOW_ID</t>
   </si>
   <si>
-    <t>2026-03-25T09:18:16.6800000Z</t>
-  </si>
-  <si>
-    <t>aa76ca808944b7f59978d267039429c4</t>
-  </si>
-  <si>
-    <t>2026-03-25T09:21:24.7930000Z</t>
-  </si>
-  <si>
-    <t>f881cdf513b4dae3400cf4c8a261a412</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.1ee7b36a20^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>2026-03-25T09:23:40.3590000Z</t>
-  </si>
-  <si>
-    <t>e91cc9722afab50e7a7862b131f90181</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.7b705a9d97^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>2026-03-25T09:25:37.1820000Z</t>
-  </si>
-  <si>
-    <t>c66cb61d5eeb614259ea4dd34ed507ce</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.a6a833871e^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>2026-03-25T09:27:17.3800000Z</t>
-  </si>
-  <si>
-    <t>f7cd02c3f6c6100acbb022ec5410c550</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.0763835870^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>2026-03-25T09:29:23.9890000Z</t>
-  </si>
-  <si>
-    <t>cd444cd506e0d405d8006028d4de605e</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.7ad59306c0^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>2026-03-25T09:31:33.6330000Z</t>
-  </si>
-  <si>
-    <t>630050bef75405d5b77c44a96b0a1786</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.10f1903f83^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>2026-03-25T09:33:31.9290000Z</t>
-  </si>
-  <si>
-    <t>4e147abe90ae0d1c631f24a743094cfd</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.5a67a2623a^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>2026-03-25T09:34:59.1100000Z</t>
-  </si>
-  <si>
-    <t>dfacd2689daef02ffd8a21080b926d24</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.f5dda23023^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
     <t>Il sistema di validazione del CDA2 non è al momento disponibile. Si prega di riprovare più tardi.</t>
   </si>
   <si>
@@ -2624,6 +2432,198 @@
   </si>
   <si>
     <t>subject_application_version: 1.0.0</t>
+  </si>
+  <si>
+    <t>2026-03-30T14:55:23.8270000Z</t>
+  </si>
+  <si>
+    <t>2026-03-30T14:59:36.9980000Z</t>
+  </si>
+  <si>
+    <t>fb8367274b3c51aab5bb6ec90049c428</t>
+  </si>
+  <si>
+    <t>2026-03-30T15:00:53.1030000Z</t>
+  </si>
+  <si>
+    <t>314b28bf60924d463be280cb9babd910</t>
+  </si>
+  <si>
+    <t>2026-03-30T15:04:07.9770000Z</t>
+  </si>
+  <si>
+    <t>9c406d3b6fe5311e66605b0f7a7e45af</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.73893a7985^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>2026-03-30T15:05:45.0690000Z</t>
+  </si>
+  <si>
+    <t>8c333e040f72886c159c217be1b79b70</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.5463d8ca36^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>2026-03-30T15:06:53.9710000Z</t>
+  </si>
+  <si>
+    <t>d8fb0915347f4adcd321bfcc9db774f7</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.26e5cbf914^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>2026-03-30T15:10:52.0610000Z</t>
+  </si>
+  <si>
+    <t>68fb89eebc19f79683e0676e9154ac97</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.ab33f43a76^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>2026-03-30T15:12:21.2310000Z</t>
+  </si>
+  <si>
+    <t>580623359c1b6f974738758ca12b899a</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.9f49eccf83^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>2026-03-30T15:14:55.9900000Z</t>
+  </si>
+  <si>
+    <t>b323dd98a84aa95269a1fe9fa7afa41f</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.bf01573272^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>2026-03-30T15:16:40.9140000Z</t>
+  </si>
+  <si>
+    <t>2cf221522a1cce6a8c2870aca881312d</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.46023735d2^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>2026-03-30T15:17:47.0290000Z</t>
+  </si>
+  <si>
+    <t>926f889b326830634380ab136a2ec460</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.27da6239ce^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>2026-03-30T15:19:29.7510000Z</t>
+  </si>
+  <si>
+    <t>1f56c5938f2aa2d85606b19e5ed2d113</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.41191a6102^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>2026-03-30T15:20:44.0610000Z</t>
+  </si>
+  <si>
+    <t>d4c1a87b08a2c0c02304aa820948d46e</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.a186d46848^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>2026-03-30T15:22:08.9850000Z</t>
+  </si>
+  <si>
+    <t>ed3538f13e500db0e5d1bd7706978ebd</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.ba969e2124^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>2026-03-30T15:23:58.0180000Z</t>
+  </si>
+  <si>
+    <t>4c427ed938a9d2061f991eead6a6a82d</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.2d51774990^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>2026-03-30T15:25:38.8020000Z</t>
+  </si>
+  <si>
+    <t>669819f489c448a7d6f2d1ab5b2ce04a</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.5ef2046673^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>2026-03-30T15:29:22.8650000Z</t>
+  </si>
+  <si>
+    <t>2356cd18ee500426ce9a14732e66513f</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.c3c8d667e0^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>2026-03-30T15:30:34.2800000Z</t>
+  </si>
+  <si>
+    <t>1d38e45dfa69c4f582ba30eb29400808</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.053b63c17f^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>66fc125153df5a3a2de2a47851e47289</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.c3ac903496^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>2026-03-30T14:57:17.9300000Z</t>
+  </si>
+  <si>
+    <t>174a9144e3ecbe6495ca7d473c60286b</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.c194494f9a^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>2026-03-30T15:33:56.1410000Z</t>
+  </si>
+  <si>
+    <t>8e9b6cbe9be7a386d2a2b524cbf3e78f</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.96bf812a7f^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>2026-03-30T15:36:15.3370000Z</t>
+  </si>
+  <si>
+    <t>ebe2d0af2409b66b2b21a8515f95a709</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.6f45d85074^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>2026-03-30T15:37:32.7630000Z</t>
+  </si>
+  <si>
+    <t>b931f81eac15e6d150a43f2936ba6c25</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.cdbbbec688^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
 </sst>
 </file>
@@ -4804,6 +4804,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:W753"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4815,7 +4816,7 @@
     <col min="6" max="6" width="13.140625" customWidth="1"/>
     <col min="7" max="7" width="35.7109375" customWidth="1"/>
     <col min="8" max="8" width="20.85546875" customWidth="1"/>
-    <col min="9" max="9" width="19.140625" customWidth="1"/>
+    <col min="9" max="9" width="34.85546875" customWidth="1"/>
     <col min="10" max="10" width="11.42578125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="25.5703125" customWidth="1"/>
     <col min="12" max="12" width="19.5703125" customWidth="1"/>
@@ -4859,7 +4860,7 @@
       </c>
       <c r="B2" s="66"/>
       <c r="C2" s="67" t="s">
-        <v>697</v>
+        <v>633</v>
       </c>
       <c r="D2" s="66"/>
       <c r="F2" s="6"/>
@@ -4887,7 +4888,7 @@
       </c>
       <c r="B3" s="69"/>
       <c r="C3" s="74" t="s">
-        <v>698</v>
+        <v>634</v>
       </c>
       <c r="D3" s="66"/>
       <c r="F3" s="6"/>
@@ -4913,7 +4914,7 @@
       <c r="A4" s="70"/>
       <c r="B4" s="71"/>
       <c r="C4" s="74" t="s">
-        <v>699</v>
+        <v>635</v>
       </c>
       <c r="D4" s="66"/>
       <c r="E4" s="4"/>
@@ -4940,7 +4941,7 @@
       <c r="A5" s="72"/>
       <c r="B5" s="73"/>
       <c r="C5" s="74" t="s">
-        <v>700</v>
+        <v>636</v>
       </c>
       <c r="D5" s="66"/>
       <c r="F5" s="6"/>
@@ -5099,7 +5100,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="10" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="27">
         <v>4</v>
       </c>
@@ -5136,7 +5137,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="11" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="29">
         <v>28</v>
       </c>
@@ -5173,7 +5174,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="12" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="29">
         <v>29</v>
       </c>
@@ -5210,7 +5211,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="13" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="29">
         <v>30</v>
       </c>
@@ -5247,7 +5248,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="14" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="29">
         <v>31</v>
       </c>
@@ -5301,16 +5302,16 @@
         <v>48</v>
       </c>
       <c r="F15" s="60">
-        <v>46106</v>
+        <v>46111</v>
       </c>
       <c r="G15" s="61" t="s">
-        <v>667</v>
+        <v>638</v>
       </c>
       <c r="H15" s="61" t="s">
-        <v>668</v>
+        <v>639</v>
       </c>
       <c r="I15" s="31" t="s">
-        <v>669</v>
+        <v>631</v>
       </c>
       <c r="J15" s="62" t="s">
         <v>75</v>
@@ -5324,7 +5325,7 @@
         <v>75</v>
       </c>
       <c r="O15" s="32" t="s">
-        <v>632</v>
+        <v>629</v>
       </c>
       <c r="P15" s="32" t="s">
         <v>541</v>
@@ -5336,7 +5337,7 @@
         <v>75</v>
       </c>
       <c r="S15" s="32" t="s">
-        <v>633</v>
+        <v>630</v>
       </c>
       <c r="T15" s="32"/>
       <c r="U15" s="33"/>
@@ -5345,7 +5346,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="16" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="29">
         <v>33</v>
       </c>
@@ -5382,7 +5383,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="17" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="29">
         <v>34</v>
       </c>
@@ -5419,7 +5420,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="18" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="29">
         <v>35</v>
       </c>
@@ -5456,7 +5457,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="19" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="29">
         <v>36</v>
       </c>
@@ -5493,7 +5494,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="20" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="29">
         <v>37</v>
       </c>
@@ -5530,7 +5531,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="21" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="29">
         <v>38</v>
       </c>
@@ -5567,7 +5568,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="22" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="29">
         <v>39</v>
       </c>
@@ -5621,16 +5622,16 @@
         <v>65</v>
       </c>
       <c r="F23" s="60">
-        <v>46106</v>
+        <v>46111</v>
       </c>
       <c r="G23" s="61" t="s">
-        <v>670</v>
+        <v>640</v>
       </c>
       <c r="H23" s="61" t="s">
-        <v>671</v>
+        <v>641</v>
       </c>
       <c r="I23" s="31" t="s">
-        <v>669</v>
+        <v>631</v>
       </c>
       <c r="J23" s="62" t="s">
         <v>75</v>
@@ -5644,7 +5645,7 @@
         <v>75</v>
       </c>
       <c r="O23" s="32" t="s">
-        <v>632</v>
+        <v>629</v>
       </c>
       <c r="P23" s="32" t="s">
         <v>541</v>
@@ -5656,7 +5657,7 @@
         <v>75</v>
       </c>
       <c r="S23" s="32" t="s">
-        <v>633</v>
+        <v>630</v>
       </c>
       <c r="T23" s="32"/>
       <c r="U23" s="33"/>
@@ -5665,7 +5666,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="24" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="29">
         <v>41</v>
       </c>
@@ -5702,7 +5703,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="25" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="29">
         <v>42</v>
       </c>
@@ -5739,7 +5740,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="26" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="29">
         <v>43</v>
       </c>
@@ -5776,7 +5777,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="27" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="29">
         <v>44</v>
       </c>
@@ -5815,7 +5816,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="28" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="29">
         <v>45</v>
       </c>
@@ -5854,7 +5855,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="29" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="29">
         <v>46</v>
       </c>
@@ -5893,7 +5894,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="30" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="29">
         <v>47</v>
       </c>
@@ -5964,7 +5965,7 @@
         <v>75</v>
       </c>
       <c r="O31" s="32" t="s">
-        <v>696</v>
+        <v>632</v>
       </c>
       <c r="P31" s="32" t="s">
         <v>541</v>
@@ -5976,7 +5977,7 @@
         <v>75</v>
       </c>
       <c r="S31" s="32" t="s">
-        <v>633</v>
+        <v>630</v>
       </c>
       <c r="T31" s="32"/>
       <c r="U31" s="33" t="s">
@@ -5987,7 +5988,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="32" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="29">
         <v>49</v>
       </c>
@@ -6026,7 +6027,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="33" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="29">
         <v>50</v>
       </c>
@@ -6065,7 +6066,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="34" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="29">
         <v>51</v>
       </c>
@@ -6104,7 +6105,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="35" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="29">
         <v>53</v>
       </c>
@@ -6141,7 +6142,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="36" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="29">
         <v>55</v>
       </c>
@@ -6178,7 +6179,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="37" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="29">
         <v>56</v>
       </c>
@@ -6215,7 +6216,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="38" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="29">
         <v>57</v>
       </c>
@@ -6252,7 +6253,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="39" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="29">
         <v>59</v>
       </c>
@@ -6289,7 +6290,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="40" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="29">
         <v>60</v>
       </c>
@@ -6326,7 +6327,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="41" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="29">
         <v>61</v>
       </c>
@@ -6363,7 +6364,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="42" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="29">
         <v>62</v>
       </c>
@@ -6400,7 +6401,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="43" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="29">
         <v>64</v>
       </c>
@@ -6437,7 +6438,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="44" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="29">
         <v>66</v>
       </c>
@@ -6474,7 +6475,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="45" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="29">
         <v>67</v>
       </c>
@@ -6511,7 +6512,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="46" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="29">
         <v>68</v>
       </c>
@@ -6548,7 +6549,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="47" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="29">
         <v>69</v>
       </c>
@@ -6585,7 +6586,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="48" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="29">
         <v>70</v>
       </c>
@@ -6622,7 +6623,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="49" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A49" s="29">
         <v>71</v>
       </c>
@@ -6659,7 +6660,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="50" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A50" s="29">
         <v>72</v>
       </c>
@@ -6696,7 +6697,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="51" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A51" s="29">
         <v>73</v>
       </c>
@@ -6733,7 +6734,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="52" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="29">
         <v>74</v>
       </c>
@@ -6770,7 +6771,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="53" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="29">
         <v>76</v>
       </c>
@@ -6807,7 +6808,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="54" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A54" s="29">
         <v>78</v>
       </c>
@@ -6844,7 +6845,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="55" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A55" s="29">
         <v>79</v>
       </c>
@@ -6881,7 +6882,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="56" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A56" s="29">
         <v>80</v>
       </c>
@@ -6918,7 +6919,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="57" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A57" s="29">
         <v>81</v>
       </c>
@@ -6955,7 +6956,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="58" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A58" s="29">
         <v>83</v>
       </c>
@@ -6992,7 +6993,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="59" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A59" s="29">
         <v>84</v>
       </c>
@@ -7029,7 +7030,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="60" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A60" s="29">
         <v>85</v>
       </c>
@@ -7066,7 +7067,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="61" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A61" s="29">
         <v>86</v>
       </c>
@@ -7103,7 +7104,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="62" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A62" s="29">
         <v>87</v>
       </c>
@@ -7140,7 +7141,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="63" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A63" s="29">
         <v>88</v>
       </c>
@@ -7177,7 +7178,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="64" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A64" s="29">
         <v>89</v>
       </c>
@@ -7214,7 +7215,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="65" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A65" s="29">
         <v>90</v>
       </c>
@@ -7251,7 +7252,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="66" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A66" s="29">
         <v>91</v>
       </c>
@@ -7288,7 +7289,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="67" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A67" s="29">
         <v>92</v>
       </c>
@@ -7325,7 +7326,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="68" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A68" s="29">
         <v>93</v>
       </c>
@@ -7362,7 +7363,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="69" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A69" s="29">
         <v>95</v>
       </c>
@@ -7399,7 +7400,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="70" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A70" s="29">
         <v>97</v>
       </c>
@@ -7436,7 +7437,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="71" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A71" s="29">
         <v>98</v>
       </c>
@@ -7473,7 +7474,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="72" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A72" s="29">
         <v>99</v>
       </c>
@@ -7510,7 +7511,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="73" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A73" s="29">
         <v>100</v>
       </c>
@@ -7547,7 +7548,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="74" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A74" s="29">
         <v>101</v>
       </c>
@@ -7584,7 +7585,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="75" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A75" s="29">
         <v>102</v>
       </c>
@@ -7621,7 +7622,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="76" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A76" s="29">
         <v>103</v>
       </c>
@@ -7658,7 +7659,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="77" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A77" s="29">
         <v>104</v>
       </c>
@@ -7695,7 +7696,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="78" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A78" s="29">
         <v>105</v>
       </c>
@@ -7732,7 +7733,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="79" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A79" s="29">
         <v>106</v>
       </c>
@@ -7769,7 +7770,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="80" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A80" s="29">
         <v>108</v>
       </c>
@@ -7806,7 +7807,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="81" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A81" s="29">
         <v>110</v>
       </c>
@@ -7843,7 +7844,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="82" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A82" s="29">
         <v>111</v>
       </c>
@@ -7880,7 +7881,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="83" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A83" s="29">
         <v>112</v>
       </c>
@@ -7917,7 +7918,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="84" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A84" s="29">
         <v>113</v>
       </c>
@@ -7954,7 +7955,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="85" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A85" s="29">
         <v>114</v>
       </c>
@@ -7991,7 +7992,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="86" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A86" s="29">
         <v>115</v>
       </c>
@@ -8028,7 +8029,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="87" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A87" s="29">
         <v>116</v>
       </c>
@@ -8065,7 +8066,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="88" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A88" s="29">
         <v>117</v>
       </c>
@@ -8102,7 +8103,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="89" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A89" s="29">
         <v>118</v>
       </c>
@@ -8139,7 +8140,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="90" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A90" s="29">
         <v>119</v>
       </c>
@@ -8176,7 +8177,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="91" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A91" s="29">
         <v>120</v>
       </c>
@@ -8213,7 +8214,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="92" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A92" s="29">
         <v>121</v>
       </c>
@@ -8250,7 +8251,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="93" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A93" s="29">
         <v>123</v>
       </c>
@@ -8287,7 +8288,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="94" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A94" s="29">
         <v>125</v>
       </c>
@@ -8324,7 +8325,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="95" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A95" s="29">
         <v>126</v>
       </c>
@@ -8361,7 +8362,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="96" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A96" s="29">
         <v>127</v>
       </c>
@@ -8398,7 +8399,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="97" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A97" s="29">
         <v>128</v>
       </c>
@@ -8435,7 +8436,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="98" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A98" s="29">
         <v>129</v>
       </c>
@@ -8472,7 +8473,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="99" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A99" s="29">
         <v>130</v>
       </c>
@@ -8509,7 +8510,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="100" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A100" s="29">
         <v>131</v>
       </c>
@@ -8546,7 +8547,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="101" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A101" s="29">
         <v>132</v>
       </c>
@@ -8583,7 +8584,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="102" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A102" s="29">
         <v>133</v>
       </c>
@@ -8620,7 +8621,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="103" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A103" s="29">
         <v>134</v>
       </c>
@@ -8657,7 +8658,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="104" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A104" s="29">
         <v>135</v>
       </c>
@@ -8694,7 +8695,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="105" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A105" s="29">
         <v>136</v>
       </c>
@@ -8731,7 +8732,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="106" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A106" s="29">
         <v>137</v>
       </c>
@@ -8768,7 +8769,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="107" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A107" s="29">
         <v>138</v>
       </c>
@@ -8805,7 +8806,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="108" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A108" s="29">
         <v>139</v>
       </c>
@@ -8842,7 +8843,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="109" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A109" s="29">
         <v>140</v>
       </c>
@@ -8879,7 +8880,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="110" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A110" s="29">
         <v>141</v>
       </c>
@@ -8916,7 +8917,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="111" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A111" s="29">
         <v>142</v>
       </c>
@@ -8953,7 +8954,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="112" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A112" s="29">
         <v>143</v>
       </c>
@@ -8990,7 +8991,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="113" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A113" s="29">
         <v>144</v>
       </c>
@@ -9027,7 +9028,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="114" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A114" s="29">
         <v>145</v>
       </c>
@@ -9064,7 +9065,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="115" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A115" s="29">
         <v>146</v>
       </c>
@@ -9118,16 +9119,16 @@
         <v>246</v>
       </c>
       <c r="F116" s="60">
-        <v>46106</v>
+        <v>46111</v>
       </c>
       <c r="G116" s="61" t="s">
-        <v>672</v>
+        <v>642</v>
       </c>
       <c r="H116" s="61" t="s">
-        <v>673</v>
+        <v>643</v>
       </c>
       <c r="I116" s="61" t="s">
-        <v>674</v>
+        <v>644</v>
       </c>
       <c r="J116" s="62" t="s">
         <v>75</v>
@@ -9141,7 +9142,7 @@
         <v>75</v>
       </c>
       <c r="O116" s="32" t="s">
-        <v>632</v>
+        <v>629</v>
       </c>
       <c r="P116" s="32" t="s">
         <v>541</v>
@@ -9153,7 +9154,7 @@
         <v>75</v>
       </c>
       <c r="S116" s="32" t="s">
-        <v>633</v>
+        <v>630</v>
       </c>
       <c r="T116" s="32"/>
       <c r="U116" s="33"/>
@@ -9179,16 +9180,16 @@
         <v>248</v>
       </c>
       <c r="F117" s="60">
-        <v>46106</v>
+        <v>46111</v>
       </c>
       <c r="G117" s="61" t="s">
-        <v>675</v>
+        <v>645</v>
       </c>
       <c r="H117" s="61" t="s">
-        <v>676</v>
+        <v>646</v>
       </c>
       <c r="I117" s="61" t="s">
-        <v>677</v>
+        <v>647</v>
       </c>
       <c r="J117" s="62" t="s">
         <v>75</v>
@@ -9202,7 +9203,7 @@
         <v>75</v>
       </c>
       <c r="O117" s="32" t="s">
-        <v>632</v>
+        <v>629</v>
       </c>
       <c r="P117" s="32" t="s">
         <v>541</v>
@@ -9214,7 +9215,7 @@
         <v>75</v>
       </c>
       <c r="S117" s="32" t="s">
-        <v>633</v>
+        <v>630</v>
       </c>
       <c r="T117" s="32"/>
       <c r="U117" s="33"/>
@@ -9240,16 +9241,16 @@
         <v>250</v>
       </c>
       <c r="F118" s="60">
-        <v>46106</v>
+        <v>46111</v>
       </c>
       <c r="G118" s="61" t="s">
-        <v>678</v>
+        <v>648</v>
       </c>
       <c r="H118" s="61" t="s">
-        <v>679</v>
+        <v>649</v>
       </c>
       <c r="I118" s="61" t="s">
-        <v>680</v>
+        <v>650</v>
       </c>
       <c r="J118" s="62" t="s">
         <v>75</v>
@@ -9263,7 +9264,7 @@
         <v>75</v>
       </c>
       <c r="O118" s="32" t="s">
-        <v>632</v>
+        <v>629</v>
       </c>
       <c r="P118" s="32" t="s">
         <v>541</v>
@@ -9275,7 +9276,7 @@
         <v>75</v>
       </c>
       <c r="S118" s="32" t="s">
-        <v>633</v>
+        <v>630</v>
       </c>
       <c r="T118" s="32"/>
       <c r="U118" s="33"/>
@@ -9301,16 +9302,16 @@
         <v>252</v>
       </c>
       <c r="F119" s="60">
-        <v>46106</v>
+        <v>46111</v>
       </c>
       <c r="G119" s="61" t="s">
-        <v>681</v>
+        <v>651</v>
       </c>
       <c r="H119" s="61" t="s">
-        <v>682</v>
+        <v>652</v>
       </c>
       <c r="I119" s="61" t="s">
-        <v>683</v>
+        <v>653</v>
       </c>
       <c r="J119" s="62" t="s">
         <v>75</v>
@@ -9324,7 +9325,7 @@
         <v>75</v>
       </c>
       <c r="O119" s="32" t="s">
-        <v>632</v>
+        <v>629</v>
       </c>
       <c r="P119" s="32" t="s">
         <v>541</v>
@@ -9336,7 +9337,7 @@
         <v>75</v>
       </c>
       <c r="S119" s="32" t="s">
-        <v>633</v>
+        <v>630</v>
       </c>
       <c r="T119" s="32"/>
       <c r="U119" s="33"/>
@@ -9362,16 +9363,16 @@
         <v>254</v>
       </c>
       <c r="F120" s="60">
-        <v>46106</v>
+        <v>46111</v>
       </c>
       <c r="G120" s="61" t="s">
-        <v>684</v>
+        <v>654</v>
       </c>
       <c r="H120" s="61" t="s">
-        <v>685</v>
+        <v>655</v>
       </c>
       <c r="I120" s="61" t="s">
-        <v>686</v>
+        <v>656</v>
       </c>
       <c r="J120" s="62" t="s">
         <v>75</v>
@@ -9385,7 +9386,7 @@
         <v>75</v>
       </c>
       <c r="O120" s="32" t="s">
-        <v>632</v>
+        <v>629</v>
       </c>
       <c r="P120" s="32" t="s">
         <v>541</v>
@@ -9397,7 +9398,7 @@
         <v>75</v>
       </c>
       <c r="S120" s="32" t="s">
-        <v>633</v>
+        <v>630</v>
       </c>
       <c r="T120" s="32"/>
       <c r="U120" s="33"/>
@@ -9423,16 +9424,16 @@
         <v>256</v>
       </c>
       <c r="F121" s="60">
-        <v>46106</v>
+        <v>46111</v>
       </c>
       <c r="G121" s="61" t="s">
-        <v>687</v>
+        <v>657</v>
       </c>
       <c r="H121" s="61" t="s">
-        <v>688</v>
+        <v>658</v>
       </c>
       <c r="I121" s="61" t="s">
-        <v>689</v>
+        <v>659</v>
       </c>
       <c r="J121" s="62" t="s">
         <v>75</v>
@@ -9446,7 +9447,7 @@
         <v>75</v>
       </c>
       <c r="O121" s="32" t="s">
-        <v>632</v>
+        <v>629</v>
       </c>
       <c r="P121" s="32" t="s">
         <v>541</v>
@@ -9458,7 +9459,7 @@
         <v>75</v>
       </c>
       <c r="S121" s="32" t="s">
-        <v>633</v>
+        <v>630</v>
       </c>
       <c r="T121" s="32"/>
       <c r="U121" s="33"/>
@@ -9484,16 +9485,16 @@
         <v>258</v>
       </c>
       <c r="F122" s="60">
-        <v>46106</v>
+        <v>46111</v>
       </c>
       <c r="G122" s="61" t="s">
-        <v>690</v>
+        <v>660</v>
       </c>
       <c r="H122" s="61" t="s">
-        <v>691</v>
+        <v>661</v>
       </c>
       <c r="I122" s="61" t="s">
-        <v>692</v>
+        <v>662</v>
       </c>
       <c r="J122" s="62" t="s">
         <v>75</v>
@@ -9507,7 +9508,7 @@
         <v>75</v>
       </c>
       <c r="O122" s="32" t="s">
-        <v>632</v>
+        <v>629</v>
       </c>
       <c r="P122" s="32" t="s">
         <v>541</v>
@@ -9519,7 +9520,7 @@
         <v>75</v>
       </c>
       <c r="S122" s="32" t="s">
-        <v>633</v>
+        <v>630</v>
       </c>
       <c r="T122" s="32"/>
       <c r="U122" s="33"/>
@@ -9545,16 +9546,16 @@
         <v>260</v>
       </c>
       <c r="F123" s="60">
-        <v>46106</v>
+        <v>46111</v>
       </c>
       <c r="G123" s="61" t="s">
-        <v>693</v>
+        <v>663</v>
       </c>
       <c r="H123" s="61" t="s">
-        <v>694</v>
+        <v>664</v>
       </c>
       <c r="I123" s="61" t="s">
-        <v>695</v>
+        <v>665</v>
       </c>
       <c r="J123" s="62" t="s">
         <v>75</v>
@@ -9568,7 +9569,7 @@
         <v>75</v>
       </c>
       <c r="O123" s="32" t="s">
-        <v>632</v>
+        <v>629</v>
       </c>
       <c r="P123" s="32" t="s">
         <v>541</v>
@@ -9580,7 +9581,7 @@
         <v>75</v>
       </c>
       <c r="S123" s="32" t="s">
-        <v>633</v>
+        <v>630</v>
       </c>
       <c r="T123" s="32"/>
       <c r="U123" s="33"/>
@@ -9606,16 +9607,16 @@
         <v>262</v>
       </c>
       <c r="F124" s="60">
-        <v>46106</v>
+        <v>46111</v>
       </c>
       <c r="G124" s="61" t="s">
-        <v>629</v>
+        <v>666</v>
       </c>
       <c r="H124" s="61" t="s">
-        <v>630</v>
+        <v>667</v>
       </c>
       <c r="I124" s="61" t="s">
-        <v>631</v>
+        <v>668</v>
       </c>
       <c r="J124" s="62" t="s">
         <v>75</v>
@@ -9629,7 +9630,7 @@
         <v>75</v>
       </c>
       <c r="O124" s="32" t="s">
-        <v>632</v>
+        <v>629</v>
       </c>
       <c r="P124" s="32" t="s">
         <v>541</v>
@@ -9641,7 +9642,7 @@
         <v>75</v>
       </c>
       <c r="S124" s="32" t="s">
-        <v>633</v>
+        <v>630</v>
       </c>
       <c r="T124" s="32"/>
       <c r="U124" s="33"/>
@@ -9667,16 +9668,16 @@
         <v>264</v>
       </c>
       <c r="F125" s="60">
-        <v>46106</v>
+        <v>46111</v>
       </c>
       <c r="G125" s="61" t="s">
-        <v>634</v>
+        <v>669</v>
       </c>
       <c r="H125" s="61" t="s">
-        <v>635</v>
+        <v>670</v>
       </c>
       <c r="I125" s="61" t="s">
-        <v>636</v>
+        <v>671</v>
       </c>
       <c r="J125" s="62" t="s">
         <v>75</v>
@@ -9690,7 +9691,7 @@
         <v>75</v>
       </c>
       <c r="O125" s="32" t="s">
-        <v>632</v>
+        <v>629</v>
       </c>
       <c r="P125" s="32" t="s">
         <v>541</v>
@@ -9702,7 +9703,7 @@
         <v>75</v>
       </c>
       <c r="S125" s="32" t="s">
-        <v>633</v>
+        <v>630</v>
       </c>
       <c r="T125" s="32"/>
       <c r="U125" s="33"/>
@@ -9728,16 +9729,16 @@
         <v>266</v>
       </c>
       <c r="F126" s="60">
-        <v>46106</v>
+        <v>46111</v>
       </c>
       <c r="G126" s="61" t="s">
-        <v>637</v>
+        <v>672</v>
       </c>
       <c r="H126" s="61" t="s">
-        <v>638</v>
+        <v>673</v>
       </c>
       <c r="I126" s="61" t="s">
-        <v>639</v>
+        <v>674</v>
       </c>
       <c r="J126" s="62" t="s">
         <v>75</v>
@@ -9751,7 +9752,7 @@
         <v>75</v>
       </c>
       <c r="O126" s="32" t="s">
-        <v>632</v>
+        <v>629</v>
       </c>
       <c r="P126" s="32" t="s">
         <v>541</v>
@@ -9763,7 +9764,7 @@
         <v>75</v>
       </c>
       <c r="S126" s="32" t="s">
-        <v>633</v>
+        <v>630</v>
       </c>
       <c r="T126" s="32"/>
       <c r="U126" s="33"/>
@@ -9789,16 +9790,16 @@
         <v>268</v>
       </c>
       <c r="F127" s="60">
-        <v>46106</v>
+        <v>46111</v>
       </c>
       <c r="G127" s="61" t="s">
-        <v>640</v>
+        <v>675</v>
       </c>
       <c r="H127" s="61" t="s">
-        <v>641</v>
+        <v>676</v>
       </c>
       <c r="I127" s="61" t="s">
-        <v>642</v>
+        <v>677</v>
       </c>
       <c r="J127" s="62" t="s">
         <v>75</v>
@@ -9812,7 +9813,7 @@
         <v>75</v>
       </c>
       <c r="O127" s="32" t="s">
-        <v>632</v>
+        <v>629</v>
       </c>
       <c r="P127" s="32" t="s">
         <v>541</v>
@@ -9824,7 +9825,7 @@
         <v>75</v>
       </c>
       <c r="S127" s="32" t="s">
-        <v>633</v>
+        <v>630</v>
       </c>
       <c r="T127" s="32"/>
       <c r="U127" s="33"/>
@@ -9850,16 +9851,16 @@
         <v>270</v>
       </c>
       <c r="F128" s="60">
-        <v>46106</v>
+        <v>46111</v>
       </c>
       <c r="G128" s="61" t="s">
-        <v>643</v>
+        <v>678</v>
       </c>
       <c r="H128" s="61" t="s">
-        <v>644</v>
+        <v>679</v>
       </c>
       <c r="I128" s="61" t="s">
-        <v>645</v>
+        <v>680</v>
       </c>
       <c r="J128" s="62" t="s">
         <v>75</v>
@@ -9873,7 +9874,7 @@
         <v>75</v>
       </c>
       <c r="O128" s="32" t="s">
-        <v>632</v>
+        <v>629</v>
       </c>
       <c r="P128" s="32" t="s">
         <v>541</v>
@@ -9885,7 +9886,7 @@
         <v>75</v>
       </c>
       <c r="S128" s="32" t="s">
-        <v>633</v>
+        <v>630</v>
       </c>
       <c r="T128" s="32"/>
       <c r="U128" s="33"/>
@@ -9911,16 +9912,16 @@
         <v>272</v>
       </c>
       <c r="F129" s="60">
-        <v>46106</v>
+        <v>46111</v>
       </c>
       <c r="G129" s="61" t="s">
-        <v>646</v>
+        <v>681</v>
       </c>
       <c r="H129" s="61" t="s">
-        <v>647</v>
+        <v>682</v>
       </c>
       <c r="I129" s="61" t="s">
-        <v>648</v>
+        <v>683</v>
       </c>
       <c r="J129" s="62" t="s">
         <v>75</v>
@@ -9934,7 +9935,7 @@
         <v>75</v>
       </c>
       <c r="O129" s="32" t="s">
-        <v>632</v>
+        <v>629</v>
       </c>
       <c r="P129" s="32" t="s">
         <v>541</v>
@@ -9946,7 +9947,7 @@
         <v>75</v>
       </c>
       <c r="S129" s="32" t="s">
-        <v>633</v>
+        <v>630</v>
       </c>
       <c r="T129" s="32"/>
       <c r="U129" s="33"/>
@@ -9972,16 +9973,16 @@
         <v>274</v>
       </c>
       <c r="F130" s="60">
-        <v>46106</v>
+        <v>46111</v>
       </c>
       <c r="G130" s="61" t="s">
-        <v>649</v>
+        <v>684</v>
       </c>
       <c r="H130" s="61" t="s">
-        <v>650</v>
+        <v>685</v>
       </c>
       <c r="I130" s="61" t="s">
-        <v>651</v>
+        <v>686</v>
       </c>
       <c r="J130" s="62" t="s">
         <v>75</v>
@@ -9995,7 +9996,7 @@
         <v>75</v>
       </c>
       <c r="O130" s="32" t="s">
-        <v>632</v>
+        <v>629</v>
       </c>
       <c r="P130" s="32" t="s">
         <v>541</v>
@@ -10007,7 +10008,7 @@
         <v>75</v>
       </c>
       <c r="S130" s="32" t="s">
-        <v>633</v>
+        <v>630</v>
       </c>
       <c r="T130" s="32"/>
       <c r="U130" s="33"/>
@@ -10016,7 +10017,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="131" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A131" s="29">
         <v>175</v>
       </c>
@@ -10053,7 +10054,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="132" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A132" s="29">
         <v>177</v>
       </c>
@@ -10090,7 +10091,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="133" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A133" s="29">
         <v>178</v>
       </c>
@@ -10127,7 +10128,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="134" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A134" s="29">
         <v>179</v>
       </c>
@@ -10164,7 +10165,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="135" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A135" s="29">
         <v>180</v>
       </c>
@@ -10201,7 +10202,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="136" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A136" s="29">
         <v>181</v>
       </c>
@@ -10238,7 +10239,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="137" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A137" s="29">
         <v>182</v>
       </c>
@@ -10275,7 +10276,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="138" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A138" s="29">
         <v>183</v>
       </c>
@@ -10312,7 +10313,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="139" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A139" s="29">
         <v>184</v>
       </c>
@@ -10349,7 +10350,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="140" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A140" s="29">
         <v>185</v>
       </c>
@@ -10386,7 +10387,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="141" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A141" s="29">
         <v>186</v>
       </c>
@@ -10423,7 +10424,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="142" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A142" s="29">
         <v>187</v>
       </c>
@@ -10460,7 +10461,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="143" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A143" s="29">
         <v>188</v>
       </c>
@@ -10497,7 +10498,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="144" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A144" s="29">
         <v>189</v>
       </c>
@@ -10534,7 +10535,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="145" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A145" s="29">
         <v>190</v>
       </c>
@@ -10571,7 +10572,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="146" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A146" s="29">
         <v>191</v>
       </c>
@@ -10608,7 +10609,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="147" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A147" s="29">
         <v>376</v>
       </c>
@@ -10645,7 +10646,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="148" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A148" s="29">
         <v>417</v>
       </c>
@@ -10682,7 +10683,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="149" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A149" s="29">
         <v>418</v>
       </c>
@@ -10719,7 +10720,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="150" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A150" s="29">
         <v>419</v>
       </c>
@@ -10756,7 +10757,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="151" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A151" s="29">
         <v>423</v>
       </c>
@@ -10793,7 +10794,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="152" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A152" s="29">
         <v>424</v>
       </c>
@@ -10830,7 +10831,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="153" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A153" s="29">
         <v>425</v>
       </c>
@@ -10869,7 +10870,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="154" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A154" s="29">
         <v>432</v>
       </c>
@@ -10906,7 +10907,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="155" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A155" s="29">
         <v>433</v>
       </c>
@@ -10943,7 +10944,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="156" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A156" s="29">
         <v>434</v>
       </c>
@@ -10980,7 +10981,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="157" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A157" s="29">
         <v>435</v>
       </c>
@@ -11017,7 +11018,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="158" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A158" s="29">
         <v>437</v>
       </c>
@@ -11054,7 +11055,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="159" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A159" s="29">
         <v>438</v>
       </c>
@@ -11091,7 +11092,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="160" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A160" s="29">
         <v>440</v>
       </c>
@@ -11128,7 +11129,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="161" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A161" s="29">
         <v>441</v>
       </c>
@@ -11165,7 +11166,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="162" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A162" s="29">
         <v>442</v>
       </c>
@@ -11202,7 +11203,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="163" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A163" s="29">
         <v>443</v>
       </c>
@@ -11256,16 +11257,16 @@
         <v>341</v>
       </c>
       <c r="F164" s="60">
-        <v>46106</v>
+        <v>46111</v>
       </c>
       <c r="G164" s="61" t="s">
-        <v>652</v>
+        <v>637</v>
       </c>
       <c r="H164" s="61" t="s">
-        <v>653</v>
+        <v>687</v>
       </c>
       <c r="I164" s="61" t="s">
-        <v>654</v>
+        <v>688</v>
       </c>
       <c r="J164" s="62" t="s">
         <v>75</v>
@@ -11303,16 +11304,16 @@
         <v>343</v>
       </c>
       <c r="F165" s="60">
-        <v>46106</v>
+        <v>46111</v>
       </c>
       <c r="G165" s="61" t="s">
-        <v>655</v>
+        <v>689</v>
       </c>
       <c r="H165" s="61" t="s">
-        <v>656</v>
+        <v>690</v>
       </c>
       <c r="I165" s="61" t="s">
-        <v>657</v>
+        <v>691</v>
       </c>
       <c r="J165" s="62" t="s">
         <v>75</v>
@@ -11333,7 +11334,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="166" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A166" s="29">
         <v>450</v>
       </c>
@@ -11370,7 +11371,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="167" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A167" s="29">
         <v>451</v>
       </c>
@@ -11407,7 +11408,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="168" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A168" s="29">
         <v>452</v>
       </c>
@@ -11444,7 +11445,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="169" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A169" s="29">
         <v>454</v>
       </c>
@@ -11481,7 +11482,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="170" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A170" s="29">
         <v>455</v>
       </c>
@@ -11518,7 +11519,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="171" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A171" s="29">
         <v>456</v>
       </c>
@@ -11555,7 +11556,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="172" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A172" s="29">
         <v>457</v>
       </c>
@@ -11592,7 +11593,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="173" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A173" s="29">
         <v>458</v>
       </c>
@@ -11629,7 +11630,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="174" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A174" s="29">
         <v>459</v>
       </c>
@@ -11666,7 +11667,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="175" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A175" s="29">
         <v>460</v>
       </c>
@@ -11720,16 +11721,16 @@
         <v>365</v>
       </c>
       <c r="F176" s="60">
-        <v>46106</v>
+        <v>46111</v>
       </c>
       <c r="G176" s="61" t="s">
-        <v>658</v>
+        <v>692</v>
       </c>
       <c r="H176" s="61" t="s">
-        <v>659</v>
+        <v>693</v>
       </c>
       <c r="I176" s="61" t="s">
-        <v>660</v>
+        <v>694</v>
       </c>
       <c r="J176" s="62" t="s">
         <v>75</v>
@@ -11743,7 +11744,7 @@
         <v>75</v>
       </c>
       <c r="O176" s="32" t="s">
-        <v>632</v>
+        <v>629</v>
       </c>
       <c r="P176" s="32" t="s">
         <v>541</v>
@@ -11755,7 +11756,7 @@
         <v>75</v>
       </c>
       <c r="S176" s="32" t="s">
-        <v>633</v>
+        <v>630</v>
       </c>
       <c r="T176" s="32"/>
       <c r="U176" s="29"/>
@@ -11764,7 +11765,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="177" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A177" s="29">
         <v>462</v>
       </c>
@@ -11801,7 +11802,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="178" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A178" s="29">
         <v>463</v>
       </c>
@@ -11838,7 +11839,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="179" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A179" s="29">
         <v>464</v>
       </c>
@@ -11875,7 +11876,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="180" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A180" s="29">
         <v>465</v>
       </c>
@@ -11912,7 +11913,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="181" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A181" s="29">
         <v>466</v>
       </c>
@@ -11949,7 +11950,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="182" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A182" s="29">
         <v>467</v>
       </c>
@@ -12003,16 +12004,16 @@
         <v>379</v>
       </c>
       <c r="F183" s="60">
-        <v>46106</v>
+        <v>46111</v>
       </c>
       <c r="G183" s="61" t="s">
-        <v>661</v>
+        <v>695</v>
       </c>
       <c r="H183" s="61" t="s">
-        <v>662</v>
+        <v>696</v>
       </c>
       <c r="I183" s="61" t="s">
-        <v>663</v>
+        <v>697</v>
       </c>
       <c r="J183" s="62" t="s">
         <v>75</v>
@@ -12026,7 +12027,7 @@
         <v>75</v>
       </c>
       <c r="O183" s="32" t="s">
-        <v>632</v>
+        <v>629</v>
       </c>
       <c r="P183" s="32" t="s">
         <v>541</v>
@@ -12038,7 +12039,7 @@
         <v>75</v>
       </c>
       <c r="S183" s="32" t="s">
-        <v>633</v>
+        <v>630</v>
       </c>
       <c r="T183" s="32"/>
       <c r="U183" s="29"/>
@@ -12047,7 +12048,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="184" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A184" s="29">
         <v>469</v>
       </c>
@@ -12084,7 +12085,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="185" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A185" s="29">
         <v>470</v>
       </c>
@@ -12121,7 +12122,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="186" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A186" s="29">
         <v>471</v>
       </c>
@@ -12158,7 +12159,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="187" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A187" s="29">
         <v>472</v>
       </c>
@@ -12195,7 +12196,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="188" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A188" s="29">
         <v>473</v>
       </c>
@@ -12232,7 +12233,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="189" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A189" s="29">
         <v>474</v>
       </c>
@@ -12286,16 +12287,16 @@
         <v>393</v>
       </c>
       <c r="F190" s="60">
-        <v>46106</v>
+        <v>46111</v>
       </c>
       <c r="G190" s="61" t="s">
-        <v>664</v>
+        <v>698</v>
       </c>
       <c r="H190" s="61" t="s">
-        <v>665</v>
+        <v>699</v>
       </c>
       <c r="I190" s="61" t="s">
-        <v>666</v>
+        <v>700</v>
       </c>
       <c r="J190" s="62" t="s">
         <v>75</v>
@@ -12309,7 +12310,7 @@
         <v>75</v>
       </c>
       <c r="O190" s="32" t="s">
-        <v>632</v>
+        <v>629</v>
       </c>
       <c r="P190" s="32" t="s">
         <v>541</v>
@@ -12321,7 +12322,7 @@
         <v>75</v>
       </c>
       <c r="S190" s="32" t="s">
-        <v>633</v>
+        <v>630</v>
       </c>
       <c r="T190" s="32"/>
       <c r="U190" s="33"/>
@@ -12330,7 +12331,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="191" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A191" s="29">
         <v>476</v>
       </c>
@@ -12367,7 +12368,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="192" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A192" s="29">
         <v>477</v>
       </c>
@@ -12404,7 +12405,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="193" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A193" s="29">
         <v>478</v>
       </c>
@@ -12441,7 +12442,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="194" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A194" s="29">
         <v>479</v>
       </c>
@@ -12478,7 +12479,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="195" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A195" s="29">
         <v>480</v>
       </c>
@@ -12515,7 +12516,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="196" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A196" s="29">
         <v>481</v>
       </c>
@@ -12552,7 +12553,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="197" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A197" s="29">
         <v>482</v>
       </c>
@@ -12589,7 +12590,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="198" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A198" s="29">
         <v>483</v>
       </c>
@@ -12626,7 +12627,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="199" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A199" s="29">
         <v>484</v>
       </c>
@@ -12663,7 +12664,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="200" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A200" s="29">
         <v>485</v>
       </c>
@@ -12700,7 +12701,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="201" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A201" s="29">
         <v>486</v>
       </c>
@@ -12737,7 +12738,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="202" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A202" s="29">
         <v>487</v>
       </c>
@@ -12774,7 +12775,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="203" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A203" s="29">
         <v>488</v>
       </c>
@@ -12811,7 +12812,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="204" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A204" s="29">
         <v>489</v>
       </c>
@@ -12848,7 +12849,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="205" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A205" s="29">
         <v>490</v>
       </c>
@@ -12887,7 +12888,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="206" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A206" s="29">
         <v>491</v>
       </c>
@@ -12924,7 +12925,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="207" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A207" s="29">
         <v>492</v>
       </c>
@@ -12961,7 +12962,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="208" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A208" s="29">
         <v>493</v>
       </c>
@@ -12998,7 +12999,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="209" spans="1:23" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:23" ht="14.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A209" s="29">
         <v>494</v>
       </c>
@@ -13035,7 +13036,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="210" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A210" s="29">
         <v>495</v>
       </c>
@@ -13072,7 +13073,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="211" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A211" s="29">
         <v>496</v>
       </c>
@@ -13109,7 +13110,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="212" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A212" s="29">
         <v>497</v>
       </c>
@@ -13146,7 +13147,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="213" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A213" s="29">
         <v>498</v>
       </c>
@@ -13183,7 +13184,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="214" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A214" s="29">
         <v>499</v>
       </c>
@@ -13220,7 +13221,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="215" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A215" s="29">
         <v>500</v>
       </c>
@@ -13257,7 +13258,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="216" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A216" s="29">
         <v>501</v>
       </c>
@@ -13294,7 +13295,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="217" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A217" s="29">
         <v>502</v>
       </c>
@@ -13331,7 +13332,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="218" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A218" s="29">
         <v>503</v>
       </c>
@@ -13368,7 +13369,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="219" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A219" s="29">
         <v>504</v>
       </c>
@@ -13405,7 +13406,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="220" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A220" s="29">
         <v>505</v>
       </c>
@@ -13444,7 +13445,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="221" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A221" s="29">
         <v>506</v>
       </c>
@@ -13481,7 +13482,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="222" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A222" s="29">
         <v>507</v>
       </c>
@@ -13518,7 +13519,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="223" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A223" s="29">
         <v>508</v>
       </c>
@@ -13555,7 +13556,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="224" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A224" s="29">
         <v>509</v>
       </c>
@@ -13592,7 +13593,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="225" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A225" s="29">
         <v>510</v>
       </c>
@@ -13629,7 +13630,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="226" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A226" s="29">
         <v>511</v>
       </c>
@@ -13666,7 +13667,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="227" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A227" s="29">
         <v>512</v>
       </c>
@@ -13703,7 +13704,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="228" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A228" s="29">
         <v>513</v>
       </c>
@@ -13740,7 +13741,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="229" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A229" s="29">
         <v>514</v>
       </c>
@@ -13777,7 +13778,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="230" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A230" s="29">
         <v>515</v>
       </c>
@@ -13814,7 +13815,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="231" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A231" s="29">
         <v>516</v>
       </c>
@@ -13851,7 +13852,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="232" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A232" s="29">
         <v>517</v>
       </c>
@@ -13888,7 +13889,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="233" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A233" s="29">
         <v>518</v>
       </c>
@@ -13925,7 +13926,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="234" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A234" s="29">
         <v>519</v>
       </c>
@@ -13962,7 +13963,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="235" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A235" s="29">
         <v>520</v>
       </c>
@@ -14001,7 +14002,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="236" spans="1:23" s="48" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:23" s="48" customFormat="1" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A236" s="41">
         <v>521</v>
       </c>
@@ -14038,7 +14039,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="237" spans="1:23" s="48" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:23" s="48" customFormat="1" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A237" s="41">
         <v>522</v>
       </c>
@@ -14075,7 +14076,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="238" spans="1:23" s="48" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:23" s="48" customFormat="1" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A238" s="41">
         <v>523</v>
       </c>
@@ -14112,7 +14113,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="239" spans="1:23" s="48" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:23" s="48" customFormat="1" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A239" s="41">
         <v>524</v>
       </c>
@@ -14149,7 +14150,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="240" spans="1:23" s="48" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:23" s="48" customFormat="1" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A240" s="41">
         <v>525</v>
       </c>
@@ -14186,7 +14187,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="241" spans="1:23" s="48" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:23" s="48" customFormat="1" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A241" s="41">
         <v>526</v>
       </c>
@@ -14223,7 +14224,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="242" spans="1:23" s="48" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:23" s="48" customFormat="1" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A242" s="41">
         <v>527</v>
       </c>
@@ -14260,7 +14261,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="243" spans="1:23" s="48" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:23" s="48" customFormat="1" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A243" s="41">
         <v>528</v>
       </c>
@@ -14297,7 +14298,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="244" spans="1:23" s="48" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:23" s="48" customFormat="1" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A244" s="41">
         <v>529</v>
       </c>
@@ -14334,7 +14335,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="245" spans="1:23" s="48" customFormat="1" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:23" s="48" customFormat="1" ht="14.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A245" s="41">
         <v>530</v>
       </c>
@@ -14373,7 +14374,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="246" spans="1:23" s="48" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:23" s="48" customFormat="1" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A246" s="41">
         <v>531</v>
       </c>
@@ -14410,7 +14411,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="247" spans="1:23" s="48" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:23" s="48" customFormat="1" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A247" s="41">
         <v>532</v>
       </c>
@@ -14447,7 +14448,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="248" spans="1:23" s="48" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:23" s="48" customFormat="1" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A248" s="41">
         <v>533</v>
       </c>
@@ -14484,7 +14485,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="249" spans="1:23" s="48" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:23" s="48" customFormat="1" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A249" s="41">
         <v>534</v>
       </c>
@@ -14521,7 +14522,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="250" spans="1:23" s="48" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:23" s="48" customFormat="1" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A250" s="41">
         <v>535</v>
       </c>
@@ -14558,7 +14559,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="251" spans="1:23" s="48" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:23" s="48" customFormat="1" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A251" s="41">
         <v>536</v>
       </c>
@@ -14595,7 +14596,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="252" spans="1:23" s="48" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:23" s="48" customFormat="1" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A252" s="41">
         <v>537</v>
       </c>
@@ -14632,7 +14633,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="253" spans="1:23" s="48" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:23" s="48" customFormat="1" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A253" s="41">
         <v>538</v>
       </c>
@@ -14669,7 +14670,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="254" spans="1:23" s="48" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:23" s="48" customFormat="1" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A254" s="41">
         <v>539</v>
       </c>
@@ -14706,7 +14707,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="255" spans="1:23" s="48" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:23" s="48" customFormat="1" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A255" s="41">
         <v>540</v>
       </c>
@@ -14743,7 +14744,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="256" spans="1:23" s="48" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:23" s="48" customFormat="1" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A256" s="41">
         <v>541</v>
       </c>
@@ -14780,7 +14781,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="257" spans="1:23" s="48" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:23" s="48" customFormat="1" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A257" s="41">
         <v>542</v>
       </c>
@@ -14817,7 +14818,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="258" spans="1:23" s="48" customFormat="1" ht="14.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:23" s="48" customFormat="1" ht="14.45" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A258" s="41">
         <v>543</v>
       </c>
@@ -14854,7 +14855,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="259" spans="1:23" s="48" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:23" s="48" customFormat="1" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A259" s="41">
         <v>544</v>
       </c>
@@ -14891,7 +14892,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="260" spans="1:23" s="48" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:23" s="48" customFormat="1" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A260" s="41">
         <v>545</v>
       </c>
@@ -14928,7 +14929,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="261" spans="1:23" s="48" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:23" s="48" customFormat="1" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A261" s="41">
         <v>546</v>
       </c>
@@ -14965,7 +14966,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="262" spans="1:23" s="48" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:23" s="48" customFormat="1" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A262" s="41">
         <v>547</v>
       </c>
@@ -15002,7 +15003,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="263" spans="1:23" s="48" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="263" spans="1:23" s="48" customFormat="1" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A263" s="41">
         <v>548</v>
       </c>
@@ -15039,7 +15040,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="264" spans="1:23" s="48" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:23" s="48" customFormat="1" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A264" s="41">
         <v>549</v>
       </c>
@@ -15076,7 +15077,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="265" spans="1:23" s="48" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:23" s="48" customFormat="1" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A265" s="41">
         <v>550</v>
       </c>
@@ -15115,7 +15116,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="266" spans="1:23" s="48" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:23" s="48" customFormat="1" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A266" s="41">
         <v>551</v>
       </c>
@@ -15152,7 +15153,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="267" spans="1:23" s="48" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:23" s="48" customFormat="1" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A267" s="41">
         <v>552</v>
       </c>
@@ -15189,7 +15190,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="268" spans="1:23" s="48" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:23" s="48" customFormat="1" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A268" s="41">
         <v>553</v>
       </c>
@@ -15226,7 +15227,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="269" spans="1:23" s="48" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:23" s="48" customFormat="1" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A269" s="41">
         <v>554</v>
       </c>
@@ -15263,7 +15264,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="270" spans="1:23" s="48" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="270" spans="1:23" s="48" customFormat="1" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A270" s="41">
         <v>555</v>
       </c>
@@ -15300,7 +15301,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="271" spans="1:23" s="48" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:23" s="48" customFormat="1" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A271" s="41">
         <v>556</v>
       </c>
@@ -15337,7 +15338,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="272" spans="1:23" s="48" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="272" spans="1:23" s="48" customFormat="1" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A272" s="41">
         <v>557</v>
       </c>
@@ -15374,7 +15375,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="273" spans="1:23" s="48" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:23" s="48" customFormat="1" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A273" s="41">
         <v>558</v>
       </c>
@@ -15411,7 +15412,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="274" spans="1:23" s="48" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:23" s="48" customFormat="1" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A274" s="41">
         <v>559</v>
       </c>
@@ -15448,7 +15449,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="275" spans="1:23" s="48" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:23" s="48" customFormat="1" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A275" s="41">
         <v>560</v>
       </c>
@@ -15485,7 +15486,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="276" spans="1:23" s="48" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="276" spans="1:23" s="48" customFormat="1" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A276" s="41">
         <v>561</v>
       </c>
@@ -15522,7 +15523,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="277" spans="1:23" s="48" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="277" spans="1:23" s="48" customFormat="1" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A277" s="41">
         <v>562</v>
       </c>
@@ -15559,7 +15560,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="278" spans="1:23" s="48" customFormat="1" ht="14.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:23" s="48" customFormat="1" ht="14.45" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A278" s="41">
         <v>563</v>
       </c>
@@ -15596,7 +15597,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="279" spans="1:23" s="48" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="279" spans="1:23" s="48" customFormat="1" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A279" s="41">
         <v>564</v>
       </c>
@@ -15633,7 +15634,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="280" spans="1:23" s="48" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="280" spans="1:23" s="48" customFormat="1" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A280" s="41">
         <v>565</v>
       </c>
@@ -15670,7 +15671,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="281" spans="1:23" s="48" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="281" spans="1:23" s="48" customFormat="1" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A281" s="41">
         <v>566</v>
       </c>
@@ -15707,7 +15708,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="282" spans="1:23" s="48" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="282" spans="1:23" s="48" customFormat="1" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A282" s="41">
         <v>567</v>
       </c>
@@ -15744,7 +15745,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="283" spans="1:23" s="48" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="283" spans="1:23" s="48" customFormat="1" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A283" s="41">
         <v>568</v>
       </c>
@@ -15781,7 +15782,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="284" spans="1:23" s="48" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="284" spans="1:23" s="48" customFormat="1" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A284" s="41">
         <v>569</v>
       </c>
@@ -15818,7 +15819,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="285" spans="1:23" s="48" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="285" spans="1:23" s="48" customFormat="1" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A285" s="41">
         <v>570</v>
       </c>
@@ -18034,7 +18035,13 @@
     <row r="752" spans="23:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="753" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <autoFilter ref="A9:W285" xr:uid="{00000000-0001-0000-0200-000000000000}"/>
+  <autoFilter ref="A9:W285" xr:uid="{00000000-0001-0000-0200-000000000000}">
+    <filterColumn colId="2">
+      <filters>
+        <filter val="RSA"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <mergeCells count="7">
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="A2:B2"/>
@@ -20378,6 +20385,27 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="a56712a3-8dfd-4688-917a-22f0cf513b89" xsi:nil="true"/>
+    <UserStoryALM xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A92AB09DCDF6014AA0D6826BF29E2C8E" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="58b13f75919cba2dcad85f84b1d5db00">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1e76d14e-d0ce-457c-8343-9b55836d9ead" xmlns:ns3="a56712a3-8dfd-4688-917a-22f0cf513b89" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a3b16ea44285e6579c272a3325f660d0" ns2:_="" ns3:_="">
     <xsd:import namespace="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
@@ -20641,42 +20669,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="a56712a3-8dfd-4688-917a-22f0cf513b89" xsi:nil="true"/>
-    <UserStoryALM xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1AD72871-87C6-44C4-AEDE-C35BE2C233EE}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
-    <ds:schemaRef ds:uri="a56712a3-8dfd-4688-917a-22f0cf513b89"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -20699,9 +20695,20 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1AD72871-87C6-44C4-AEDE-C35BE2C233EE}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
+    <ds:schemaRef ds:uri="a56712a3-8dfd-4688-917a-22f0cf513b89"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>